<commit_message>
fix: harden China Southern batch booking import
</commit_message>
<xml_diff>
--- a/documents/china_southern_air/南航订舱模板.xlsx
+++ b/documents/china_southern_air/南航订舱模板.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="南航批量订舱" sheetId="1" r:id="R21d5ea8e0a6e43e7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="南航批量订舱" sheetId="1" r:id="Rd20524f6f14c467d"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -99,7 +99,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="27">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -150,6 +150,18 @@
     </x:xf>
     <x:xf numFmtId="203" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="202" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="203" fontId="3" fillId="4" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="1" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="3" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -368,7 +380,7 @@
     <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="17" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="12" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
@@ -376,676 +388,692 @@
   </x:cols>
   <x:sheetData>
     <x:row r="1" ht="42" customHeight="1">
-      <x:c r="A1" s="4" t="str">
+      <x:c r="A1" s="25" t="str">
         <x:v>南航订舱模板</x:v>
       </x:c>
-      <x:c r="B1" s="4"/>
-      <x:c r="C1" s="4"/>
-      <x:c r="D1" s="4"/>
-      <x:c r="E1" s="4"/>
-      <x:c r="F1" s="4"/>
-      <x:c r="G1" s="4"/>
-      <x:c r="H1" s="4"/>
-      <x:c r="I1" s="4"/>
-      <x:c r="J1" s="4"/>
-      <x:c r="K1" s="4"/>
-      <x:c r="L1" s="4"/>
-      <x:c r="M1" s="4"/>
-      <x:c r="N1" s="4"/>
-      <x:c r="O1" s="4"/>
-      <x:c r="P1" s="4"/>
-      <x:c r="Q1" s="4"/>
-      <x:c r="R1" s="4"/>
-      <x:c r="S1" s="4"/>
-      <x:c r="T1" s="4"/>
+      <x:c r="B1" s="25"/>
+      <x:c r="C1" s="25"/>
+      <x:c r="D1" s="25"/>
+      <x:c r="E1" s="25"/>
+      <x:c r="F1" s="25"/>
+      <x:c r="G1" s="25"/>
+      <x:c r="H1" s="25"/>
+      <x:c r="I1" s="25"/>
+      <x:c r="J1" s="25"/>
+      <x:c r="K1" s="25"/>
+      <x:c r="L1" s="25"/>
+      <x:c r="M1" s="25"/>
+      <x:c r="N1" s="25"/>
+      <x:c r="O1" s="25"/>
+      <x:c r="P1" s="25"/>
+      <x:c r="Q1" s="25"/>
+      <x:c r="R1" s="25"/>
+      <x:c r="S1" s="25"/>
+      <x:c r="T1" s="25"/>
     </x:row>
     <x:row r="2" ht="25" customHeight="1">
-      <x:c r="A2" s="10" t="str">
+      <x:c r="A2" s="26" t="str">
         <x:v>序号</x:v>
       </x:c>
-      <x:c r="B2" s="10" t="str">
+      <x:c r="B2" s="26" t="str">
         <x:v>始发站</x:v>
       </x:c>
-      <x:c r="C2" s="10" t="str">
+      <x:c r="C2" s="26" t="str">
         <x:v>到达站</x:v>
       </x:c>
-      <x:c r="D2" s="10" t="str">
+      <x:c r="D2" s="26" t="str">
         <x:v>航班日期</x:v>
       </x:c>
-      <x:c r="E2" s="10" t="str">
+      <x:c r="E2" s="26" t="str">
         <x:v>客户名称</x:v>
       </x:c>
-      <x:c r="F2" s="10" t="str">
+      <x:c r="F2" s="26" t="str">
         <x:v>货物类型</x:v>
       </x:c>
-      <x:c r="G2" s="10" t="str">
+      <x:c r="G2" s="26" t="str">
         <x:v>货物代码</x:v>
       </x:c>
-      <x:c r="H2" s="10" t="str">
+      <x:c r="H2" s="26" t="str">
         <x:v>航班号</x:v>
       </x:c>
-      <x:c r="I2" s="10" t="str">
+      <x:c r="I2" s="26" t="str">
         <x:v>宽体机订舱备注</x:v>
       </x:c>
-      <x:c r="J2" s="10" t="str">
+      <x:c r="J2" s="26" t="str">
         <x:v>窄体机订舱备注</x:v>
       </x:c>
-      <x:c r="K2" s="10" t="str">
+      <x:c r="K2" s="26" t="str">
         <x:v>货物名称</x:v>
       </x:c>
-      <x:c r="L2" s="10" t="str">
+      <x:c r="L2" s="26" t="str">
         <x:v>件数</x:v>
       </x:c>
-      <x:c r="M2" s="10" t="str">
+      <x:c r="M2" s="26" t="str">
         <x:v>重量(kg)</x:v>
       </x:c>
-      <x:c r="N2" s="10" t="str">
+      <x:c r="N2" s="26" t="str">
         <x:v>产品名称</x:v>
       </x:c>
-      <x:c r="O2" s="10" t="str">
+      <x:c r="O2" s="26" t="str">
         <x:v>超规货</x:v>
       </x:c>
-      <x:c r="P2" s="10" t="str">
-        <x:v>特货码</x:v>
-      </x:c>
-      <x:c r="Q2" s="10" t="str">
+      <x:c r="P2" s="26" t="str">
+        <x:v>特货码（多个特货码用/隔开）</x:v>
+      </x:c>
+      <x:c r="Q2" s="26" t="str">
         <x:v>订舱体积</x:v>
       </x:c>
-      <x:c r="R2" s="10" t="str">
+      <x:c r="R2" s="26" t="str">
         <x:v>储运注意事项</x:v>
       </x:c>
-      <x:c r="S2" s="10" t="str">
+      <x:c r="S2" s="26" t="str">
         <x:v>无隐含危险品</x:v>
       </x:c>
-      <x:c r="T2" s="10" t="str">
+      <x:c r="T2" s="26" t="str">
         <x:v>出港货邮处理费选项</x:v>
       </x:c>
     </x:row>
     <x:row r="3" ht="25" customHeight="1">
-      <x:c r="A3" s="10"/>
-      <x:c r="B3" s="10"/>
-      <x:c r="C3" s="10"/>
-      <x:c r="D3" s="10"/>
-      <x:c r="E3" s="10"/>
-      <x:c r="F3" s="10"/>
-      <x:c r="G3" s="10"/>
-      <x:c r="H3" s="10"/>
-      <x:c r="I3" s="10"/>
-      <x:c r="J3" s="10"/>
-      <x:c r="K3" s="10"/>
-      <x:c r="L3" s="10"/>
-      <x:c r="M3" s="10"/>
-      <x:c r="N3" s="10"/>
-      <x:c r="O3" s="10"/>
-      <x:c r="P3" s="10"/>
-      <x:c r="Q3" s="10"/>
-      <x:c r="R3" s="10"/>
-      <x:c r="S3" s="10"/>
-      <x:c r="T3" s="10"/>
+      <x:c r="A3" s="26"/>
+      <x:c r="B3" s="26"/>
+      <x:c r="C3" s="26"/>
+      <x:c r="D3" s="26"/>
+      <x:c r="E3" s="26"/>
+      <x:c r="F3" s="26"/>
+      <x:c r="G3" s="26"/>
+      <x:c r="H3" s="26"/>
+      <x:c r="I3" s="26"/>
+      <x:c r="J3" s="26"/>
+      <x:c r="K3" s="26"/>
+      <x:c r="L3" s="26"/>
+      <x:c r="M3" s="26"/>
+      <x:c r="N3" s="26"/>
+      <x:c r="O3" s="26"/>
+      <x:c r="P3" s="26"/>
+      <x:c r="Q3" s="26"/>
+      <x:c r="R3" s="26"/>
+      <x:c r="S3" s="26"/>
+      <x:c r="T3" s="26"/>
     </x:row>
     <x:row r="4" ht="24" customHeight="1">
-      <x:c r="A4" s="15" t="n">
+      <x:c r="A4" s="18" t="str">
         <x:v>1</x:v>
       </x:c>
       <x:c r="B4" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C4" s="18"/>
-      <x:c r="D4" s="17"/>
-      <x:c r="E4" s="19"/>
-      <x:c r="F4" s="19"/>
-      <x:c r="G4" s="19"/>
-      <x:c r="H4" s="19"/>
-      <x:c r="I4" s="19"/>
-      <x:c r="J4" s="19"/>
-      <x:c r="K4" s="19"/>
-      <x:c r="L4" s="20"/>
-      <x:c r="M4" s="21"/>
-      <x:c r="N4" s="19"/>
+      <x:c r="D4" s="18"/>
+      <x:c r="E4" s="18"/>
+      <x:c r="F4" s="18"/>
+      <x:c r="G4" s="18"/>
+      <x:c r="H4" s="18"/>
+      <x:c r="I4" s="18"/>
+      <x:c r="J4" s="18"/>
+      <x:c r="K4" s="18"/>
+      <x:c r="L4" s="18"/>
+      <x:c r="M4" s="18"/>
+      <x:c r="N4" s="18"/>
       <x:c r="O4" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P4" s="19"/>
-      <x:c r="Q4" s="22"/>
-      <x:c r="R4" s="19"/>
+      <x:c r="P4" s="18"/>
+      <x:c r="Q4" s="18"/>
+      <x:c r="R4" s="18"/>
       <x:c r="S4" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T4" s="18"/>
     </x:row>
     <x:row r="5" ht="24" customHeight="1">
-      <x:c r="A5" s="15" t="n">
+      <x:c r="A5" s="18" t="str">
         <x:v>2</x:v>
       </x:c>
       <x:c r="B5" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C5" s="18"/>
-      <x:c r="D5" s="17"/>
-      <x:c r="E5" s="19"/>
-      <x:c r="F5" s="19"/>
-      <x:c r="G5" s="19"/>
-      <x:c r="H5" s="19"/>
-      <x:c r="I5" s="19"/>
-      <x:c r="J5" s="19"/>
-      <x:c r="K5" s="19"/>
-      <x:c r="L5" s="20"/>
-      <x:c r="M5" s="21"/>
-      <x:c r="N5" s="19"/>
+      <x:c r="D5" s="18"/>
+      <x:c r="E5" s="18"/>
+      <x:c r="F5" s="18"/>
+      <x:c r="G5" s="18"/>
+      <x:c r="H5" s="18"/>
+      <x:c r="I5" s="18"/>
+      <x:c r="J5" s="18"/>
+      <x:c r="K5" s="18"/>
+      <x:c r="L5" s="18"/>
+      <x:c r="M5" s="18"/>
+      <x:c r="N5" s="18"/>
       <x:c r="O5" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P5" s="19"/>
-      <x:c r="Q5" s="22"/>
-      <x:c r="R5" s="19"/>
+      <x:c r="P5" s="18"/>
+      <x:c r="Q5" s="18"/>
+      <x:c r="R5" s="18"/>
       <x:c r="S5" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T5" s="18"/>
     </x:row>
     <x:row r="6" ht="24" customHeight="1">
-      <x:c r="A6" s="15" t="n">
+      <x:c r="A6" s="18" t="str">
         <x:v>3</x:v>
       </x:c>
       <x:c r="B6" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C6" s="18"/>
-      <x:c r="D6" s="17"/>
-      <x:c r="E6" s="19"/>
-      <x:c r="F6" s="19"/>
-      <x:c r="G6" s="19"/>
-      <x:c r="H6" s="19"/>
-      <x:c r="I6" s="19"/>
-      <x:c r="J6" s="19"/>
-      <x:c r="K6" s="19"/>
-      <x:c r="L6" s="20"/>
-      <x:c r="M6" s="21"/>
-      <x:c r="N6" s="19"/>
+      <x:c r="D6" s="18"/>
+      <x:c r="E6" s="18"/>
+      <x:c r="F6" s="18"/>
+      <x:c r="G6" s="18"/>
+      <x:c r="H6" s="18"/>
+      <x:c r="I6" s="18"/>
+      <x:c r="J6" s="18"/>
+      <x:c r="K6" s="18"/>
+      <x:c r="L6" s="18"/>
+      <x:c r="M6" s="18"/>
+      <x:c r="N6" s="18"/>
       <x:c r="O6" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P6" s="19"/>
-      <x:c r="Q6" s="22"/>
-      <x:c r="R6" s="19"/>
+      <x:c r="P6" s="18"/>
+      <x:c r="Q6" s="18"/>
+      <x:c r="R6" s="18"/>
       <x:c r="S6" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T6" s="18"/>
     </x:row>
     <x:row r="7" ht="24" customHeight="1">
-      <x:c r="A7" s="15" t="n">
+      <x:c r="A7" s="18" t="str">
         <x:v>4</x:v>
       </x:c>
       <x:c r="B7" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C7" s="18"/>
-      <x:c r="D7" s="17"/>
-      <x:c r="E7" s="19"/>
-      <x:c r="F7" s="19"/>
-      <x:c r="G7" s="19"/>
-      <x:c r="H7" s="19"/>
-      <x:c r="I7" s="19"/>
-      <x:c r="J7" s="19"/>
-      <x:c r="K7" s="19"/>
-      <x:c r="L7" s="20"/>
-      <x:c r="M7" s="21"/>
-      <x:c r="N7" s="19"/>
+      <x:c r="D7" s="18"/>
+      <x:c r="E7" s="18"/>
+      <x:c r="F7" s="18"/>
+      <x:c r="G7" s="18"/>
+      <x:c r="H7" s="18"/>
+      <x:c r="I7" s="18"/>
+      <x:c r="J7" s="18"/>
+      <x:c r="K7" s="18"/>
+      <x:c r="L7" s="18"/>
+      <x:c r="M7" s="18"/>
+      <x:c r="N7" s="18"/>
       <x:c r="O7" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P7" s="19"/>
-      <x:c r="Q7" s="22"/>
-      <x:c r="R7" s="19"/>
+      <x:c r="P7" s="18"/>
+      <x:c r="Q7" s="18"/>
+      <x:c r="R7" s="18"/>
       <x:c r="S7" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T7" s="18"/>
     </x:row>
     <x:row r="8" ht="24" customHeight="1">
-      <x:c r="A8" s="15" t="n">
+      <x:c r="A8" s="18" t="str">
         <x:v>5</x:v>
       </x:c>
       <x:c r="B8" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C8" s="18"/>
-      <x:c r="D8" s="17"/>
-      <x:c r="E8" s="19"/>
-      <x:c r="F8" s="19"/>
-      <x:c r="G8" s="19"/>
-      <x:c r="H8" s="19"/>
-      <x:c r="I8" s="19"/>
-      <x:c r="J8" s="19"/>
-      <x:c r="K8" s="19"/>
-      <x:c r="L8" s="20"/>
-      <x:c r="M8" s="21"/>
-      <x:c r="N8" s="19"/>
+      <x:c r="D8" s="18"/>
+      <x:c r="E8" s="18"/>
+      <x:c r="F8" s="18"/>
+      <x:c r="G8" s="18"/>
+      <x:c r="H8" s="18"/>
+      <x:c r="I8" s="18"/>
+      <x:c r="J8" s="18"/>
+      <x:c r="K8" s="18"/>
+      <x:c r="L8" s="18"/>
+      <x:c r="M8" s="18"/>
+      <x:c r="N8" s="18"/>
       <x:c r="O8" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P8" s="19"/>
-      <x:c r="Q8" s="22"/>
-      <x:c r="R8" s="19"/>
+      <x:c r="P8" s="18"/>
+      <x:c r="Q8" s="18"/>
+      <x:c r="R8" s="18"/>
       <x:c r="S8" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T8" s="18"/>
     </x:row>
     <x:row r="9" ht="24" customHeight="1">
-      <x:c r="A9" s="15" t="n">
+      <x:c r="A9" s="18" t="str">
         <x:v>6</x:v>
       </x:c>
       <x:c r="B9" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C9" s="18"/>
-      <x:c r="D9" s="17"/>
-      <x:c r="E9" s="19"/>
-      <x:c r="F9" s="19"/>
-      <x:c r="G9" s="19"/>
-      <x:c r="H9" s="19"/>
-      <x:c r="I9" s="19"/>
-      <x:c r="J9" s="19"/>
-      <x:c r="K9" s="19"/>
-      <x:c r="L9" s="20"/>
-      <x:c r="M9" s="21"/>
-      <x:c r="N9" s="19"/>
+      <x:c r="D9" s="18"/>
+      <x:c r="E9" s="18"/>
+      <x:c r="F9" s="18"/>
+      <x:c r="G9" s="18"/>
+      <x:c r="H9" s="18"/>
+      <x:c r="I9" s="18"/>
+      <x:c r="J9" s="18"/>
+      <x:c r="K9" s="18"/>
+      <x:c r="L9" s="18"/>
+      <x:c r="M9" s="18"/>
+      <x:c r="N9" s="18"/>
       <x:c r="O9" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P9" s="19"/>
-      <x:c r="Q9" s="22"/>
-      <x:c r="R9" s="19"/>
+      <x:c r="P9" s="18"/>
+      <x:c r="Q9" s="18"/>
+      <x:c r="R9" s="18"/>
       <x:c r="S9" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T9" s="18"/>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
-      <x:c r="A10" s="15" t="n">
+      <x:c r="A10" s="18" t="str">
         <x:v>7</x:v>
       </x:c>
       <x:c r="B10" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C10" s="18"/>
-      <x:c r="D10" s="17"/>
-      <x:c r="E10" s="19"/>
-      <x:c r="F10" s="19"/>
-      <x:c r="G10" s="19"/>
-      <x:c r="H10" s="19"/>
-      <x:c r="I10" s="19"/>
-      <x:c r="J10" s="19"/>
-      <x:c r="K10" s="19"/>
-      <x:c r="L10" s="20"/>
-      <x:c r="M10" s="21"/>
-      <x:c r="N10" s="19"/>
+      <x:c r="D10" s="18"/>
+      <x:c r="E10" s="18"/>
+      <x:c r="F10" s="18"/>
+      <x:c r="G10" s="18"/>
+      <x:c r="H10" s="18"/>
+      <x:c r="I10" s="18"/>
+      <x:c r="J10" s="18"/>
+      <x:c r="K10" s="18"/>
+      <x:c r="L10" s="18"/>
+      <x:c r="M10" s="18"/>
+      <x:c r="N10" s="18"/>
       <x:c r="O10" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P10" s="19"/>
-      <x:c r="Q10" s="22"/>
-      <x:c r="R10" s="19"/>
+      <x:c r="P10" s="18"/>
+      <x:c r="Q10" s="18"/>
+      <x:c r="R10" s="18"/>
       <x:c r="S10" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T10" s="18"/>
     </x:row>
     <x:row r="11" ht="24" customHeight="1">
-      <x:c r="A11" s="15" t="n">
+      <x:c r="A11" s="18" t="str">
         <x:v>8</x:v>
       </x:c>
       <x:c r="B11" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C11" s="18"/>
-      <x:c r="D11" s="17"/>
-      <x:c r="E11" s="19"/>
-      <x:c r="F11" s="19"/>
-      <x:c r="G11" s="19"/>
-      <x:c r="H11" s="19"/>
-      <x:c r="I11" s="19"/>
-      <x:c r="J11" s="19"/>
-      <x:c r="K11" s="19"/>
-      <x:c r="L11" s="20"/>
-      <x:c r="M11" s="21"/>
-      <x:c r="N11" s="19"/>
+      <x:c r="D11" s="18"/>
+      <x:c r="E11" s="18"/>
+      <x:c r="F11" s="18"/>
+      <x:c r="G11" s="18"/>
+      <x:c r="H11" s="18"/>
+      <x:c r="I11" s="18"/>
+      <x:c r="J11" s="18"/>
+      <x:c r="K11" s="18"/>
+      <x:c r="L11" s="18"/>
+      <x:c r="M11" s="18"/>
+      <x:c r="N11" s="18"/>
       <x:c r="O11" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P11" s="19"/>
-      <x:c r="Q11" s="22"/>
-      <x:c r="R11" s="19"/>
+      <x:c r="P11" s="18"/>
+      <x:c r="Q11" s="18"/>
+      <x:c r="R11" s="18"/>
       <x:c r="S11" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T11" s="18"/>
     </x:row>
     <x:row r="12" ht="24" customHeight="1">
-      <x:c r="A12" s="15" t="n">
+      <x:c r="A12" s="18" t="str">
         <x:v>9</x:v>
       </x:c>
       <x:c r="B12" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C12" s="18"/>
-      <x:c r="D12" s="17"/>
-      <x:c r="E12" s="19"/>
-      <x:c r="F12" s="19"/>
-      <x:c r="G12" s="19"/>
-      <x:c r="H12" s="19"/>
-      <x:c r="I12" s="19"/>
-      <x:c r="J12" s="19"/>
-      <x:c r="K12" s="19"/>
-      <x:c r="L12" s="20"/>
-      <x:c r="M12" s="21"/>
-      <x:c r="N12" s="19"/>
+      <x:c r="D12" s="18"/>
+      <x:c r="E12" s="18"/>
+      <x:c r="F12" s="18"/>
+      <x:c r="G12" s="18"/>
+      <x:c r="H12" s="18"/>
+      <x:c r="I12" s="18"/>
+      <x:c r="J12" s="18"/>
+      <x:c r="K12" s="18"/>
+      <x:c r="L12" s="18"/>
+      <x:c r="M12" s="18"/>
+      <x:c r="N12" s="18"/>
       <x:c r="O12" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P12" s="19"/>
-      <x:c r="Q12" s="22"/>
-      <x:c r="R12" s="19"/>
+      <x:c r="P12" s="18"/>
+      <x:c r="Q12" s="18"/>
+      <x:c r="R12" s="18"/>
       <x:c r="S12" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T12" s="18"/>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
-      <x:c r="A13" s="15" t="n">
+      <x:c r="A13" s="18" t="str">
         <x:v>10</x:v>
       </x:c>
       <x:c r="B13" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C13" s="18"/>
-      <x:c r="D13" s="17"/>
-      <x:c r="E13" s="19"/>
-      <x:c r="F13" s="19"/>
-      <x:c r="G13" s="19"/>
-      <x:c r="H13" s="19"/>
-      <x:c r="I13" s="19"/>
-      <x:c r="J13" s="19"/>
-      <x:c r="K13" s="19"/>
-      <x:c r="L13" s="20"/>
-      <x:c r="M13" s="21"/>
-      <x:c r="N13" s="19"/>
+      <x:c r="D13" s="18"/>
+      <x:c r="E13" s="18"/>
+      <x:c r="F13" s="18"/>
+      <x:c r="G13" s="18"/>
+      <x:c r="H13" s="18"/>
+      <x:c r="I13" s="18"/>
+      <x:c r="J13" s="18"/>
+      <x:c r="K13" s="18"/>
+      <x:c r="L13" s="18"/>
+      <x:c r="M13" s="18"/>
+      <x:c r="N13" s="18"/>
       <x:c r="O13" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P13" s="19"/>
-      <x:c r="Q13" s="22"/>
-      <x:c r="R13" s="19"/>
+      <x:c r="P13" s="18"/>
+      <x:c r="Q13" s="18"/>
+      <x:c r="R13" s="18"/>
       <x:c r="S13" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T13" s="18"/>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
-      <x:c r="A14" s="15" t="n">
+      <x:c r="A14" s="18" t="str">
         <x:v>11</x:v>
       </x:c>
       <x:c r="B14" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C14" s="18"/>
-      <x:c r="D14" s="17"/>
-      <x:c r="E14" s="19"/>
-      <x:c r="F14" s="19"/>
-      <x:c r="G14" s="19"/>
-      <x:c r="H14" s="19"/>
-      <x:c r="I14" s="19"/>
-      <x:c r="J14" s="19"/>
-      <x:c r="K14" s="19"/>
-      <x:c r="L14" s="20"/>
-      <x:c r="M14" s="21"/>
-      <x:c r="N14" s="19"/>
+      <x:c r="D14" s="18"/>
+      <x:c r="E14" s="18"/>
+      <x:c r="F14" s="18"/>
+      <x:c r="G14" s="18"/>
+      <x:c r="H14" s="18"/>
+      <x:c r="I14" s="18"/>
+      <x:c r="J14" s="18"/>
+      <x:c r="K14" s="18"/>
+      <x:c r="L14" s="18"/>
+      <x:c r="M14" s="18"/>
+      <x:c r="N14" s="18"/>
       <x:c r="O14" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P14" s="19"/>
-      <x:c r="Q14" s="22"/>
-      <x:c r="R14" s="19"/>
+      <x:c r="P14" s="18"/>
+      <x:c r="Q14" s="18"/>
+      <x:c r="R14" s="18"/>
       <x:c r="S14" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T14" s="18"/>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
-      <x:c r="A15" s="15" t="n">
+      <x:c r="A15" s="18" t="str">
         <x:v>12</x:v>
       </x:c>
       <x:c r="B15" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C15" s="18"/>
-      <x:c r="D15" s="17"/>
-      <x:c r="E15" s="19"/>
-      <x:c r="F15" s="19"/>
-      <x:c r="G15" s="19"/>
-      <x:c r="H15" s="19"/>
-      <x:c r="I15" s="19"/>
-      <x:c r="J15" s="19"/>
-      <x:c r="K15" s="19"/>
-      <x:c r="L15" s="20"/>
-      <x:c r="M15" s="21"/>
-      <x:c r="N15" s="19"/>
+      <x:c r="D15" s="18"/>
+      <x:c r="E15" s="18"/>
+      <x:c r="F15" s="18"/>
+      <x:c r="G15" s="18"/>
+      <x:c r="H15" s="18"/>
+      <x:c r="I15" s="18"/>
+      <x:c r="J15" s="18"/>
+      <x:c r="K15" s="18"/>
+      <x:c r="L15" s="18"/>
+      <x:c r="M15" s="18"/>
+      <x:c r="N15" s="18"/>
       <x:c r="O15" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P15" s="19"/>
-      <x:c r="Q15" s="22"/>
-      <x:c r="R15" s="19"/>
+      <x:c r="P15" s="18"/>
+      <x:c r="Q15" s="18"/>
+      <x:c r="R15" s="18"/>
       <x:c r="S15" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T15" s="18"/>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
-      <x:c r="A16" s="15" t="n">
+      <x:c r="A16" s="18" t="str">
         <x:v>13</x:v>
       </x:c>
       <x:c r="B16" s="18" t="str">
         <x:v>SZX</x:v>
       </x:c>
       <x:c r="C16" s="18"/>
-      <x:c r="D16" s="17"/>
-      <x:c r="E16" s="19"/>
-      <x:c r="F16" s="19"/>
-      <x:c r="G16" s="19"/>
-      <x:c r="H16" s="19"/>
-      <x:c r="I16" s="19"/>
-      <x:c r="J16" s="19"/>
-      <x:c r="K16" s="19"/>
-      <x:c r="L16" s="20"/>
-      <x:c r="M16" s="21"/>
-      <x:c r="N16" s="19"/>
+      <x:c r="D16" s="18"/>
+      <x:c r="E16" s="18"/>
+      <x:c r="F16" s="18"/>
+      <x:c r="G16" s="18"/>
+      <x:c r="H16" s="18"/>
+      <x:c r="I16" s="18"/>
+      <x:c r="J16" s="18"/>
+      <x:c r="K16" s="18"/>
+      <x:c r="L16" s="18"/>
+      <x:c r="M16" s="18"/>
+      <x:c r="N16" s="18"/>
       <x:c r="O16" s="18" t="str">
         <x:v>否</x:v>
       </x:c>
-      <x:c r="P16" s="19"/>
-      <x:c r="Q16" s="22"/>
-      <x:c r="R16" s="19"/>
+      <x:c r="P16" s="18"/>
+      <x:c r="Q16" s="18"/>
+      <x:c r="R16" s="18"/>
       <x:c r="S16" s="18" t="str">
         <x:v>是</x:v>
       </x:c>
       <x:c r="T16" s="18"/>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
-      <x:c r="A17" s="15"/>
+      <x:c r="A17" s="18" t="str">
+        <x:v>14</x:v>
+      </x:c>
       <x:c r="B17" s="18"/>
       <x:c r="C17" s="18"/>
-      <x:c r="D17" s="17"/>
-      <x:c r="E17" s="19"/>
-      <x:c r="F17" s="19"/>
-      <x:c r="G17" s="19"/>
-      <x:c r="H17" s="19"/>
-      <x:c r="I17" s="19"/>
-      <x:c r="J17" s="19"/>
-      <x:c r="K17" s="19"/>
-      <x:c r="L17" s="20"/>
-      <x:c r="M17" s="21"/>
-      <x:c r="N17" s="19"/>
+      <x:c r="D17" s="18"/>
+      <x:c r="E17" s="18"/>
+      <x:c r="F17" s="18"/>
+      <x:c r="G17" s="18"/>
+      <x:c r="H17" s="18"/>
+      <x:c r="I17" s="18"/>
+      <x:c r="J17" s="18"/>
+      <x:c r="K17" s="18"/>
+      <x:c r="L17" s="18"/>
+      <x:c r="M17" s="18"/>
+      <x:c r="N17" s="18"/>
       <x:c r="O17" s="18"/>
-      <x:c r="P17" s="19"/>
-      <x:c r="Q17" s="22"/>
-      <x:c r="R17" s="19"/>
+      <x:c r="P17" s="18"/>
+      <x:c r="Q17" s="18"/>
+      <x:c r="R17" s="18"/>
       <x:c r="S17" s="18"/>
       <x:c r="T17" s="18"/>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
-      <x:c r="A18" s="15"/>
+      <x:c r="A18" s="18" t="str">
+        <x:v>15</x:v>
+      </x:c>
       <x:c r="B18" s="18"/>
       <x:c r="C18" s="18"/>
-      <x:c r="D18" s="17"/>
-      <x:c r="E18" s="19"/>
-      <x:c r="F18" s="19"/>
-      <x:c r="G18" s="19"/>
-      <x:c r="H18" s="19"/>
-      <x:c r="I18" s="19"/>
-      <x:c r="J18" s="19"/>
-      <x:c r="K18" s="19"/>
-      <x:c r="L18" s="20"/>
-      <x:c r="M18" s="21"/>
-      <x:c r="N18" s="19"/>
+      <x:c r="D18" s="18"/>
+      <x:c r="E18" s="18"/>
+      <x:c r="F18" s="18"/>
+      <x:c r="G18" s="18"/>
+      <x:c r="H18" s="18"/>
+      <x:c r="I18" s="18"/>
+      <x:c r="J18" s="18"/>
+      <x:c r="K18" s="18"/>
+      <x:c r="L18" s="18"/>
+      <x:c r="M18" s="18"/>
+      <x:c r="N18" s="18"/>
       <x:c r="O18" s="18"/>
-      <x:c r="P18" s="19"/>
-      <x:c r="Q18" s="22"/>
-      <x:c r="R18" s="19"/>
+      <x:c r="P18" s="18"/>
+      <x:c r="Q18" s="18"/>
+      <x:c r="R18" s="18"/>
       <x:c r="S18" s="18"/>
       <x:c r="T18" s="18"/>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
-      <x:c r="A19" s="15"/>
+      <x:c r="A19" s="18" t="str">
+        <x:v>16</x:v>
+      </x:c>
       <x:c r="B19" s="18"/>
       <x:c r="C19" s="18"/>
-      <x:c r="D19" s="17"/>
-      <x:c r="E19" s="19"/>
-      <x:c r="F19" s="19"/>
-      <x:c r="G19" s="19"/>
-      <x:c r="H19" s="19"/>
-      <x:c r="I19" s="19"/>
-      <x:c r="J19" s="19"/>
-      <x:c r="K19" s="19"/>
-      <x:c r="L19" s="20"/>
-      <x:c r="M19" s="21"/>
-      <x:c r="N19" s="19"/>
+      <x:c r="D19" s="18"/>
+      <x:c r="E19" s="18"/>
+      <x:c r="F19" s="18"/>
+      <x:c r="G19" s="18"/>
+      <x:c r="H19" s="18"/>
+      <x:c r="I19" s="18"/>
+      <x:c r="J19" s="18"/>
+      <x:c r="K19" s="18"/>
+      <x:c r="L19" s="18"/>
+      <x:c r="M19" s="18"/>
+      <x:c r="N19" s="18"/>
       <x:c r="O19" s="18"/>
-      <x:c r="P19" s="19"/>
-      <x:c r="Q19" s="22"/>
-      <x:c r="R19" s="19"/>
+      <x:c r="P19" s="18"/>
+      <x:c r="Q19" s="18"/>
+      <x:c r="R19" s="18"/>
       <x:c r="S19" s="18"/>
       <x:c r="T19" s="18"/>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
-      <x:c r="A20" s="15"/>
+      <x:c r="A20" s="18" t="str">
+        <x:v>17</x:v>
+      </x:c>
       <x:c r="B20" s="18"/>
       <x:c r="C20" s="18"/>
-      <x:c r="D20" s="17"/>
-      <x:c r="E20" s="19"/>
-      <x:c r="F20" s="19"/>
-      <x:c r="G20" s="19"/>
-      <x:c r="H20" s="19"/>
-      <x:c r="I20" s="19"/>
-      <x:c r="J20" s="19"/>
-      <x:c r="K20" s="19"/>
-      <x:c r="L20" s="20"/>
-      <x:c r="M20" s="21"/>
-      <x:c r="N20" s="19"/>
+      <x:c r="D20" s="18"/>
+      <x:c r="E20" s="18"/>
+      <x:c r="F20" s="18"/>
+      <x:c r="G20" s="18"/>
+      <x:c r="H20" s="18"/>
+      <x:c r="I20" s="18"/>
+      <x:c r="J20" s="18"/>
+      <x:c r="K20" s="18"/>
+      <x:c r="L20" s="18"/>
+      <x:c r="M20" s="18"/>
+      <x:c r="N20" s="18"/>
       <x:c r="O20" s="18"/>
-      <x:c r="P20" s="19"/>
-      <x:c r="Q20" s="22"/>
-      <x:c r="R20" s="19"/>
+      <x:c r="P20" s="18"/>
+      <x:c r="Q20" s="18"/>
+      <x:c r="R20" s="18"/>
       <x:c r="S20" s="18"/>
       <x:c r="T20" s="18"/>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
-      <x:c r="A21" s="15"/>
+      <x:c r="A21" s="18" t="str">
+        <x:v>18</x:v>
+      </x:c>
       <x:c r="B21" s="18"/>
       <x:c r="C21" s="18"/>
-      <x:c r="D21" s="17"/>
-      <x:c r="E21" s="19"/>
-      <x:c r="F21" s="19"/>
-      <x:c r="G21" s="19"/>
-      <x:c r="H21" s="19"/>
-      <x:c r="I21" s="19"/>
-      <x:c r="J21" s="19"/>
-      <x:c r="K21" s="19"/>
-      <x:c r="L21" s="20"/>
-      <x:c r="M21" s="21"/>
-      <x:c r="N21" s="19"/>
+      <x:c r="D21" s="18"/>
+      <x:c r="E21" s="18"/>
+      <x:c r="F21" s="18"/>
+      <x:c r="G21" s="18"/>
+      <x:c r="H21" s="18"/>
+      <x:c r="I21" s="18"/>
+      <x:c r="J21" s="18"/>
+      <x:c r="K21" s="18"/>
+      <x:c r="L21" s="18"/>
+      <x:c r="M21" s="18"/>
+      <x:c r="N21" s="18"/>
       <x:c r="O21" s="18"/>
-      <x:c r="P21" s="19"/>
-      <x:c r="Q21" s="22"/>
-      <x:c r="R21" s="19"/>
+      <x:c r="P21" s="18"/>
+      <x:c r="Q21" s="18"/>
+      <x:c r="R21" s="18"/>
       <x:c r="S21" s="18"/>
       <x:c r="T21" s="18"/>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
-      <x:c r="A22" s="15"/>
+      <x:c r="A22" s="18" t="str">
+        <x:v>19</x:v>
+      </x:c>
       <x:c r="B22" s="18"/>
       <x:c r="C22" s="18"/>
-      <x:c r="D22" s="17"/>
-      <x:c r="E22" s="19"/>
-      <x:c r="F22" s="19"/>
-      <x:c r="G22" s="19"/>
-      <x:c r="H22" s="19"/>
-      <x:c r="I22" s="19"/>
-      <x:c r="J22" s="19"/>
-      <x:c r="K22" s="19"/>
-      <x:c r="L22" s="20"/>
-      <x:c r="M22" s="21"/>
-      <x:c r="N22" s="19"/>
+      <x:c r="D22" s="18"/>
+      <x:c r="E22" s="18"/>
+      <x:c r="F22" s="18"/>
+      <x:c r="G22" s="18"/>
+      <x:c r="H22" s="18"/>
+      <x:c r="I22" s="18"/>
+      <x:c r="J22" s="18"/>
+      <x:c r="K22" s="18"/>
+      <x:c r="L22" s="18"/>
+      <x:c r="M22" s="18"/>
+      <x:c r="N22" s="18"/>
       <x:c r="O22" s="18"/>
-      <x:c r="P22" s="19"/>
-      <x:c r="Q22" s="22"/>
-      <x:c r="R22" s="19"/>
+      <x:c r="P22" s="18"/>
+      <x:c r="Q22" s="18"/>
+      <x:c r="R22" s="18"/>
       <x:c r="S22" s="18"/>
       <x:c r="T22" s="18"/>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
-      <x:c r="A23" s="15"/>
+      <x:c r="A23" s="18" t="str">
+        <x:v>20</x:v>
+      </x:c>
       <x:c r="B23" s="18"/>
       <x:c r="C23" s="18"/>
-      <x:c r="D23" s="17"/>
-      <x:c r="E23" s="19"/>
-      <x:c r="F23" s="19"/>
-      <x:c r="G23" s="19"/>
-      <x:c r="H23" s="19"/>
-      <x:c r="I23" s="19"/>
-      <x:c r="J23" s="19"/>
-      <x:c r="K23" s="19"/>
-      <x:c r="L23" s="20"/>
-      <x:c r="M23" s="21"/>
-      <x:c r="N23" s="19"/>
+      <x:c r="D23" s="18"/>
+      <x:c r="E23" s="18"/>
+      <x:c r="F23" s="18"/>
+      <x:c r="G23" s="18"/>
+      <x:c r="H23" s="18"/>
+      <x:c r="I23" s="18"/>
+      <x:c r="J23" s="18"/>
+      <x:c r="K23" s="18"/>
+      <x:c r="L23" s="18"/>
+      <x:c r="M23" s="18"/>
+      <x:c r="N23" s="18"/>
       <x:c r="O23" s="18"/>
-      <x:c r="P23" s="19"/>
-      <x:c r="Q23" s="22"/>
-      <x:c r="R23" s="19"/>
+      <x:c r="P23" s="18"/>
+      <x:c r="Q23" s="18"/>
+      <x:c r="R23" s="18"/>
       <x:c r="S23" s="18"/>
       <x:c r="T23" s="18"/>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
-      <x:c r="A24" s="15"/>
+      <x:c r="A24" s="18" t="str">
+        <x:v>21</x:v>
+      </x:c>
       <x:c r="B24" s="18"/>
       <x:c r="C24" s="18"/>
-      <x:c r="D24" s="17"/>
-      <x:c r="E24" s="19"/>
-      <x:c r="F24" s="19"/>
-      <x:c r="G24" s="19"/>
-      <x:c r="H24" s="19"/>
-      <x:c r="I24" s="19"/>
-      <x:c r="J24" s="19"/>
-      <x:c r="K24" s="19"/>
-      <x:c r="L24" s="20"/>
-      <x:c r="M24" s="21"/>
-      <x:c r="N24" s="19"/>
+      <x:c r="D24" s="18"/>
+      <x:c r="E24" s="18"/>
+      <x:c r="F24" s="18"/>
+      <x:c r="G24" s="18"/>
+      <x:c r="H24" s="18"/>
+      <x:c r="I24" s="18"/>
+      <x:c r="J24" s="18"/>
+      <x:c r="K24" s="18"/>
+      <x:c r="L24" s="18"/>
+      <x:c r="M24" s="18"/>
+      <x:c r="N24" s="18"/>
       <x:c r="O24" s="18"/>
-      <x:c r="P24" s="19"/>
-      <x:c r="Q24" s="22"/>
-      <x:c r="R24" s="19"/>
+      <x:c r="P24" s="18"/>
+      <x:c r="Q24" s="18"/>
+      <x:c r="R24" s="18"/>
       <x:c r="S24" s="18"/>
       <x:c r="T24" s="18"/>
     </x:row>

</xml_diff>

<commit_message>
fix: normalize China Southern special cargo codes
</commit_message>
<xml_diff>
--- a/documents/china_southern_air/南航订舱模板.xlsx
+++ b/documents/china_southern_air/南航订舱模板.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="南航批量订舱" sheetId="1" r:id="Rd20524f6f14c467d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="南航批量订舱" sheetId="1" r:id="Rd0c505b2b48045a0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -380,7 +380,7 @@
     <x:col min="13" max="13" width="12" hidden="0" customWidth="1"/>
     <x:col min="14" max="14" width="14" hidden="0" customWidth="1"/>
     <x:col min="15" max="15" width="10" hidden="0" customWidth="1"/>
-    <x:col min="16" max="16" width="25" hidden="0" customWidth="1"/>
+    <x:col min="16" max="16" width="26" hidden="0" customWidth="1"/>
     <x:col min="17" max="17" width="12" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="14" hidden="0" customWidth="1"/>
@@ -458,7 +458,7 @@
         <x:v>超规货</x:v>
       </x:c>
       <x:c r="P2" s="26" t="str">
-        <x:v>特货码（多个特货码用/隔开）</x:v>
+        <x:v>特货码（多个用英文逗号隔开）</x:v>
       </x:c>
       <x:c r="Q2" s="26" t="str">
         <x:v>订舱体积</x:v>

</xml_diff>